<commit_message>
COMP-751 updating excel template to include compliance finding
</commit_message>
<xml_diff>
--- a/compliance-api/src/compliance_api/services/report/ceb_template.xlsx
+++ b/compliance-api/src/compliance_api/services/report/ceb_template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30006"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30015"/>
   <workbookPr hidePivotFieldList="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tayalee/Desktop/Excel pivot tables_forfeedback/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="208" documentId="13_ncr:1_{0AC415D9-D733-894D-B4A0-A67D0E09A217}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E137CF07-F6FD-464A-A35B-3675555BCA3B}"/>
+  <xr:revisionPtr revIDLastSave="226" documentId="13_ncr:1_{0AC415D9-D733-894D-B4A0-A67D0E09A217}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7783AECA-6842-4DC1-A2AF-E967C7476B32}"/>
   <bookViews>
     <workbookView xWindow="35080" yWindow="1540" windowWidth="34560" windowHeight="20260" firstSheet="3" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,9 +20,9 @@
   </sheets>
   <calcPr calcId="191028"/>
   <pivotCaches>
-    <pivotCache cacheId="1011" r:id="rId5"/>
-    <pivotCache cacheId="1018" r:id="rId6"/>
-    <pivotCache cacheId="1024" r:id="rId7"/>
+    <pivotCache cacheId="1430" r:id="rId5"/>
+    <pivotCache cacheId="1437" r:id="rId6"/>
+    <pivotCache cacheId="1441" r:id="rId7"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -117,7 +117,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="K2" authorId="0" shapeId="0" xr:uid="{54A4951F-359C-2B4C-B5F0-8D56596EFF78}">
+    <comment ref="L2" authorId="0" shapeId="0" xr:uid="{54A4951F-359C-2B4C-B5F0-8D56596EFF78}">
       <text>
         <r>
           <rPr>
@@ -187,7 +187,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="28">
   <si>
     <t>IR Number</t>
   </si>
@@ -264,13 +264,13 @@
     <t>Column Labels</t>
   </si>
   <si>
+    <t>(blank)</t>
+  </si>
+  <si>
+    <t>Grand Total</t>
+  </si>
+  <si>
     <t>Count of Enforcement Action</t>
-  </si>
-  <si>
-    <t>(blank)</t>
-  </si>
-  <si>
-    <t>Grand Total</t>
   </si>
 </sst>
 </file>
@@ -355,6 +355,27 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.39997558519241921"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.39997558519241921"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.39997558519241921"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
           <bgColor theme="3"/>
         </patternFill>
       </fill>
@@ -394,27 +415,6 @@
         </patternFill>
       </fill>
     </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="4" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="4" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="4" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -435,23 +435,51 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshOnLoad="1" refreshedBy="Excel Services" refreshedDate="46129.602462847222" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="1" xr:uid="{9A655F1F-804E-4F57-A400-987732F35DAD}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshOnLoad="1" refreshedBy="Excel Services" refreshedDate="46133.494440046299" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="1" xr:uid="{E508D2FB-1B6C-4B04-92EF-07C92A3B7FD7}">
   <cacheSource type="worksheet">
-    <worksheetSource name="Inspections"/>
+    <worksheetSource name="Requirements"/>
   </cacheSource>
-  <cacheFields count="8">
+  <cacheFields count="16">
     <cacheField name="IR Number" numFmtId="0">
       <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
     </cacheField>
+    <cacheField name="Topic" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="Summary" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
     <cacheField name="IR Progress" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="Project Name" numFmtId="0">
       <sharedItems containsNonDate="0" containsString="0" containsBlank="1" count="1">
         <m/>
       </sharedItems>
     </cacheField>
-    <cacheField name="Project Name" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
-    </cacheField>
     <cacheField name="Project Type" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1" count="1">
+        <m/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Compliance Finding" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1" count="1">
+        <m/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Enforcement Action" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="Enforcement Status" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="Enforcement Document Number" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="Condition Number" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="Requirement Source" numFmtId="0">
       <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
     </cacheField>
     <cacheField name="IR Issuance Date" numFmtId="0">
@@ -476,11 +504,11 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshOnLoad="1" refreshedBy="Excel Services" refreshedDate="46129.602462847222" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="1" xr:uid="{3DC42666-42A1-448D-A623-A82BC44CBAFC}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshOnLoad="1" refreshedBy="Excel Services" refreshedDate="46133.494440046299" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="1" xr:uid="{3DC42666-42A1-448D-A623-A82BC44CBAFC}">
   <cacheSource type="worksheet">
     <worksheetSource name="Enforcements"/>
   </cacheSource>
-  <cacheFields count="13">
+  <cacheFields count="14">
     <cacheField name="IR Number" numFmtId="0">
       <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
     </cacheField>
@@ -493,6 +521,9 @@
       </sharedItems>
     </cacheField>
     <cacheField name="Project Type" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="Compliance Finding" numFmtId="0">
       <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
     </cacheField>
     <cacheField name="Enforcement Action" numFmtId="0">
@@ -538,51 +569,23 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshOnLoad="1" refreshedBy="Excel Services" refreshedDate="46129.602462847222" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="1" xr:uid="{E508D2FB-1B6C-4B04-92EF-07C92A3B7FD7}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshOnLoad="1" refreshedBy="Excel Services" refreshedDate="46133.494440046299" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="1" xr:uid="{9A655F1F-804E-4F57-A400-987732F35DAD}">
   <cacheSource type="worksheet">
-    <worksheetSource name="Requirements"/>
+    <worksheetSource name="Inspections"/>
   </cacheSource>
-  <cacheFields count="16">
+  <cacheFields count="8">
     <cacheField name="IR Number" numFmtId="0">
       <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
     </cacheField>
-    <cacheField name="Topic" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
-    </cacheField>
-    <cacheField name="Summary" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
-    </cacheField>
     <cacheField name="IR Progress" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
-    </cacheField>
-    <cacheField name="Project Name" numFmtId="0">
       <sharedItems containsNonDate="0" containsString="0" containsBlank="1" count="1">
         <m/>
       </sharedItems>
     </cacheField>
+    <cacheField name="Project Name" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
     <cacheField name="Project Type" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1" count="1">
-        <m/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="Compliance Finding" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1" count="1">
-        <m/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="Enforcement Action" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
-    </cacheField>
-    <cacheField name="Enforcement Status" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
-    </cacheField>
-    <cacheField name="Enforcement Document Number" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
-    </cacheField>
-    <cacheField name="Condition Number" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
-    </cacheField>
-    <cacheField name="Requirement Source" numFmtId="0">
       <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
     </cacheField>
     <cacheField name="IR Issuance Date" numFmtId="0">
@@ -607,101 +610,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{F3646FCF-C206-4361-8690-240132D1671E}" name="PivotTable24" cacheId="1018" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="K4:M9" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
-  <pivotFields count="13">
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="2">
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" dataField="1" showAll="0">
-      <items count="2">
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField axis="axisCol" showAll="0">
-      <items count="2">
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="2">
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="3">
-    <field x="2"/>
-    <field x="4"/>
-    <field x="6"/>
-  </rowFields>
-  <rowItems count="4">
-    <i>
-      <x/>
-    </i>
-    <i r="1">
-      <x/>
-    </i>
-    <i r="2">
-      <x/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colFields count="1">
-    <field x="5"/>
-  </colFields>
-  <colItems count="2">
-    <i>
-      <x/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Count of Enforcement Action" fld="4" subtotal="count" baseField="0" baseItem="0"/>
-  </dataFields>
-  <formats count="3">
-    <format dxfId="7">
-      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="8">
-      <pivotArea field="5" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
-    </format>
-    <format dxfId="9">
-      <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
-    </format>
-  </formats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{3A2CB471-5EA6-4127-A467-E8F5D9596452}" name="PivotTable23" cacheId="1024" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{3A2CB471-5EA6-4127-A467-E8F5D9596452}" name="PivotTable23" cacheId="1430" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="E4:G8" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="16">
     <pivotField showAll="0"/>
@@ -766,15 +675,6 @@
     <dataField name="Count of Summary" fld="2" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="6">
-    <format dxfId="1">
-      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="2">
-      <pivotArea field="6" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
-    </format>
-    <format dxfId="3">
-      <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
-    </format>
     <format dxfId="4">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
@@ -782,6 +682,15 @@
       <pivotArea field="6" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
     <format dxfId="6">
+      <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="7">
+      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="8">
+      <pivotArea field="6" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
+    </format>
+    <format dxfId="9">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -797,8 +706,8 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{DE23F307-6508-443D-9D35-8D0EAB9E4958}" name="PivotTable22" cacheId="1011" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{DE23F307-6508-443D-9D35-8D0EAB9E4958}" name="PivotTable22" cacheId="1441" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="B4:C6" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="8">
     <pivotField dataField="1" showAll="0"/>
@@ -844,6 +753,101 @@
 </pivotTableDefinition>
 </file>
 
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{F3646FCF-C206-4361-8690-240132D1671E}" name="PivotTable24" cacheId="1437" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="L6:N11" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="14">
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="2">
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" dataField="1" showAll="0">
+      <items count="2">
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisCol" showAll="0">
+      <items count="2">
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="2">
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="3">
+    <field x="2"/>
+    <field x="5"/>
+    <field x="7"/>
+  </rowFields>
+  <rowItems count="4">
+    <i>
+      <x/>
+    </i>
+    <i r="1">
+      <x/>
+    </i>
+    <i r="2">
+      <x/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="6"/>
+  </colFields>
+  <colItems count="2">
+    <i>
+      <x/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Count of Enforcement Action" fld="5" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <formats count="3">
+    <format dxfId="1">
+      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="2">
+      <pivotArea field="6" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
+    </format>
+    <format dxfId="3">
+      <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+    </format>
+  </formats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{25A5AAF5-465E-40DA-80D8-7D63F24C71CF}" name="Inspections" displayName="Inspections" ref="A1:H2" totalsRowShown="0">
   <autoFilter ref="A1:H2" xr:uid="{25A5AAF5-465E-40DA-80D8-7D63F24C71CF}"/>
@@ -887,13 +891,14 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{BB558FF6-8E88-4B8C-85F0-A9AC1F3494E1}" name="Enforcements" displayName="Enforcements" ref="A1:M2" totalsRowShown="0">
-  <autoFilter ref="A1:M2" xr:uid="{BB558FF6-8E88-4B8C-85F0-A9AC1F3494E1}"/>
-  <tableColumns count="13">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{BB558FF6-8E88-4B8C-85F0-A9AC1F3494E1}" name="Enforcements" displayName="Enforcements" ref="A1:N2" totalsRowShown="0">
+  <autoFilter ref="A1:N2" xr:uid="{BB558FF6-8E88-4B8C-85F0-A9AC1F3494E1}"/>
+  <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{002DF4D9-2342-465C-AFA9-D19EC440D92D}" name="IR Number"/>
     <tableColumn id="2" xr3:uid="{121E0AA8-E00F-4A87-B2E8-39B632F930A5}" name="IR Progress"/>
     <tableColumn id="3" xr3:uid="{6A40920A-25DB-4945-B49C-37E79325503F}" name="Project Name"/>
     <tableColumn id="4" xr3:uid="{BFB4DB6B-0FE0-47F2-B2D1-38090A00D902}" name="Project Type"/>
+    <tableColumn id="14" xr3:uid="{0C33F754-7EED-4DC1-A065-4630AFD7D772}" name="Compliance Finding"/>
     <tableColumn id="5" xr3:uid="{EB406C39-C322-4377-9490-1E84DC84279E}" name="Enforcement Action"/>
     <tableColumn id="6" xr3:uid="{5C25DE55-141D-4A51-AF8A-3E0C7590A8B3}" name="Enforcement Status"/>
     <tableColumn id="7" xr3:uid="{6D85C97C-DB2A-45AC-8D60-9844F03DFAE0}" name="Enforcement Document Number"/>
@@ -1331,7 +1336,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FBAE1F1F-8658-4E77-804F-851BEEBDB0CE}">
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:N1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="2" width="14.5703125" customWidth="1"/>
@@ -1348,7 +1353,7 @@
     <col min="13" max="13" width="13.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13">
+    <row r="1" spans="1:14">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1362,30 +1367,33 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F1" t="s">
         <v>11</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>12</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>13</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>4</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>5</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>6</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>7</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>16</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -1399,21 +1407,21 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C3DA8C2-D460-3E49-93A1-0DC80ABEB419}">
-  <dimension ref="B2:M33"/>
+  <dimension ref="B2:N33"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="14.28515625" customWidth="1"/>
     <col min="3" max="3" width="19.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12.140625" customWidth="1"/>
-    <col min="5" max="5" width="20.140625" customWidth="1"/>
+    <col min="5" max="5" width="18" customWidth="1"/>
     <col min="6" max="6" width="17.28515625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="11.7109375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="12" customWidth="1"/>
     <col min="9" max="9" width="27.5703125" customWidth="1"/>
     <col min="10" max="10" width="17.28515625" customWidth="1"/>
-    <col min="11" max="11" width="31.85546875" customWidth="1"/>
-    <col min="12" max="12" width="24" customWidth="1"/>
-    <col min="13" max="13" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.7109375" customWidth="1"/>
+    <col min="12" max="12" width="17.28515625" customWidth="1"/>
+    <col min="13" max="13" width="11.7109375" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="14" customWidth="1"/>
     <col min="15" max="15" width="13.140625" customWidth="1"/>
     <col min="16" max="16" width="15.7109375" customWidth="1"/>
@@ -1485,18 +1493,18 @@
     <col min="125" max="125" width="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:13">
+    <row r="2" spans="2:14">
       <c r="B2" t="s">
         <v>18</v>
       </c>
       <c r="E2" t="s">
         <v>19</v>
       </c>
-      <c r="K2" t="s">
+      <c r="L2" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="2:13">
+    <row r="4" spans="2:14">
       <c r="B4" s="1" t="s">
         <v>21</v>
       </c>
@@ -1510,84 +1518,88 @@
         <v>24</v>
       </c>
       <c r="G4" s="4"/>
-      <c r="K4" s="4" t="s">
+    </row>
+    <row r="5" spans="2:14">
+      <c r="B5" s="2" t="s">
         <v>25</v>
-      </c>
-      <c r="L4" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="M4" s="4"/>
-    </row>
-    <row r="5" spans="2:13">
-      <c r="B5" s="2" t="s">
-        <v>26</v>
       </c>
       <c r="C5" s="6"/>
       <c r="E5" s="1" t="s">
         <v>21</v>
       </c>
       <c r="F5" t="s">
+        <v>25</v>
+      </c>
+      <c r="G5" t="s">
         <v>26</v>
       </c>
-      <c r="G5" t="s">
-        <v>27</v>
-      </c>
-      <c r="K5" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="L5" t="s">
+    </row>
+    <row r="6" spans="2:14">
+      <c r="B6" s="2" t="s">
         <v>26</v>
-      </c>
-      <c r="M5" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="6" spans="2:13">
-      <c r="B6" s="2" t="s">
-        <v>27</v>
       </c>
       <c r="C6" s="6"/>
       <c r="E6" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F6" s="6"/>
       <c r="G6" s="6"/>
-      <c r="K6" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="L6" s="6"/>
-      <c r="M6" s="6"/>
+      <c r="L6" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="M6" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="N6" s="4"/>
     </row>
-    <row r="7" spans="2:13">
+    <row r="7" spans="2:14">
       <c r="E7" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F7" s="6"/>
       <c r="G7" s="6"/>
-      <c r="K7" s="3" t="s">
+      <c r="L7" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="M7" t="s">
+        <v>25</v>
+      </c>
+      <c r="N7" t="s">
         <v>26</v>
       </c>
-      <c r="L7" s="6"/>
-      <c r="M7" s="6"/>
     </row>
-    <row r="8" spans="2:13">
+    <row r="8" spans="2:14">
       <c r="E8" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F8" s="6"/>
       <c r="G8" s="6"/>
-      <c r="K8" s="5" t="s">
+      <c r="L8" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M8" s="6"/>
+      <c r="N8" s="6"/>
+    </row>
+    <row r="9" spans="2:14">
+      <c r="L9" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="M9" s="6"/>
+      <c r="N9" s="6"/>
+    </row>
+    <row r="10" spans="2:14">
+      <c r="L10" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="M10" s="6"/>
+      <c r="N10" s="6"/>
+    </row>
+    <row r="11" spans="2:14">
+      <c r="L11" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="L8" s="6"/>
-      <c r="M8" s="6"/>
-    </row>
-    <row r="9" spans="2:13">
-      <c r="K9" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="L9" s="6"/>
-      <c r="M9" s="6"/>
+      <c r="M11" s="6"/>
+      <c r="N11" s="6"/>
     </row>
     <row r="33" spans="12:12"/>
   </sheetData>

</xml_diff>

<commit_message>
COMP-751 adding filters to pivot tables
</commit_message>
<xml_diff>
--- a/compliance-api/src/compliance_api/services/report/ceb_template.xlsx
+++ b/compliance-api/src/compliance_api/services/report/ceb_template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30006"/>
-  <workbookPr hidePivotFieldList="1"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30015"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tayalee/Desktop/Excel pivot tables_forfeedback/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="208" documentId="13_ncr:1_{0AC415D9-D733-894D-B4A0-A67D0E09A217}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E137CF07-F6FD-464A-A35B-3675555BCA3B}"/>
+  <xr:revisionPtr revIDLastSave="230" documentId="13_ncr:1_{0AC415D9-D733-894D-B4A0-A67D0E09A217}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9698F4B5-39DB-4005-8176-674D149EF680}"/>
   <bookViews>
     <workbookView xWindow="35080" yWindow="1540" windowWidth="34560" windowHeight="20260" firstSheet="3" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,9 +20,9 @@
   </sheets>
   <calcPr calcId="191028"/>
   <pivotCaches>
-    <pivotCache cacheId="1011" r:id="rId5"/>
-    <pivotCache cacheId="1018" r:id="rId6"/>
-    <pivotCache cacheId="1024" r:id="rId7"/>
+    <pivotCache cacheId="1510" r:id="rId5"/>
+    <pivotCache cacheId="1518" r:id="rId6"/>
+    <pivotCache cacheId="1522" r:id="rId7"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -117,7 +117,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="K2" authorId="0" shapeId="0" xr:uid="{54A4951F-359C-2B4C-B5F0-8D56596EFF78}">
+    <comment ref="L2" authorId="0" shapeId="0" xr:uid="{54A4951F-359C-2B4C-B5F0-8D56596EFF78}">
       <text>
         <r>
           <rPr>
@@ -187,7 +187,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="29">
   <si>
     <t>IR Number</t>
   </si>
@@ -264,13 +264,16 @@
     <t>Column Labels</t>
   </si>
   <si>
+    <t>(All)</t>
+  </si>
+  <si>
+    <t>(blank)</t>
+  </si>
+  <si>
+    <t>Grand Total</t>
+  </si>
+  <si>
     <t>Count of Enforcement Action</t>
-  </si>
-  <si>
-    <t>(blank)</t>
-  </si>
-  <si>
-    <t>Grand Total</t>
   </si>
 </sst>
 </file>
@@ -355,6 +358,27 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.39997558519241921"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.39997558519241921"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.39997558519241921"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
           <bgColor theme="3"/>
         </patternFill>
       </fill>
@@ -394,27 +418,6 @@
         </patternFill>
       </fill>
     </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="4" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="4" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="4" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -435,23 +438,51 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshOnLoad="1" refreshedBy="Excel Services" refreshedDate="46129.602462847222" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="1" xr:uid="{9A655F1F-804E-4F57-A400-987732F35DAD}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshOnLoad="1" refreshedBy="Excel Services" refreshedDate="46134.432263078706" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="1" xr:uid="{E508D2FB-1B6C-4B04-92EF-07C92A3B7FD7}">
   <cacheSource type="worksheet">
-    <worksheetSource name="Inspections"/>
+    <worksheetSource name="Requirements"/>
   </cacheSource>
-  <cacheFields count="8">
+  <cacheFields count="16">
     <cacheField name="IR Number" numFmtId="0">
       <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
     </cacheField>
+    <cacheField name="Topic" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="Summary" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
     <cacheField name="IR Progress" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="Project Name" numFmtId="0">
       <sharedItems containsNonDate="0" containsString="0" containsBlank="1" count="1">
         <m/>
       </sharedItems>
     </cacheField>
-    <cacheField name="Project Name" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
-    </cacheField>
     <cacheField name="Project Type" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1" count="1">
+        <m/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Compliance Finding" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1" count="1">
+        <m/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Enforcement Action" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="Enforcement Status" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="Enforcement Document Number" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="Condition Number" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="Requirement Source" numFmtId="0">
       <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
     </cacheField>
     <cacheField name="IR Issuance Date" numFmtId="0">
@@ -476,11 +507,11 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshOnLoad="1" refreshedBy="Excel Services" refreshedDate="46129.602462847222" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="1" xr:uid="{3DC42666-42A1-448D-A623-A82BC44CBAFC}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshOnLoad="1" refreshedBy="Excel Services" refreshedDate="46134.432263194445" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="1" xr:uid="{3DC42666-42A1-448D-A623-A82BC44CBAFC}">
   <cacheSource type="worksheet">
     <worksheetSource name="Enforcements"/>
   </cacheSource>
-  <cacheFields count="13">
+  <cacheFields count="14">
     <cacheField name="IR Number" numFmtId="0">
       <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
     </cacheField>
@@ -494,6 +525,11 @@
     </cacheField>
     <cacheField name="Project Type" numFmtId="0">
       <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="Compliance Finding" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1" count="1">
+        <m/>
+      </sharedItems>
     </cacheField>
     <cacheField name="Enforcement Action" numFmtId="0">
       <sharedItems containsNonDate="0" containsString="0" containsBlank="1" count="1">
@@ -538,51 +574,23 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshOnLoad="1" refreshedBy="Excel Services" refreshedDate="46129.602462847222" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="1" xr:uid="{E508D2FB-1B6C-4B04-92EF-07C92A3B7FD7}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshOnLoad="1" refreshedBy="Excel Services" refreshedDate="46134.432263194445" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="1" xr:uid="{9A655F1F-804E-4F57-A400-987732F35DAD}">
   <cacheSource type="worksheet">
-    <worksheetSource name="Requirements"/>
+    <worksheetSource name="Inspections"/>
   </cacheSource>
-  <cacheFields count="16">
+  <cacheFields count="8">
     <cacheField name="IR Number" numFmtId="0">
       <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
     </cacheField>
-    <cacheField name="Topic" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
-    </cacheField>
-    <cacheField name="Summary" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
-    </cacheField>
     <cacheField name="IR Progress" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
-    </cacheField>
-    <cacheField name="Project Name" numFmtId="0">
       <sharedItems containsNonDate="0" containsString="0" containsBlank="1" count="1">
         <m/>
       </sharedItems>
     </cacheField>
+    <cacheField name="Project Name" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
     <cacheField name="Project Type" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1" count="1">
-        <m/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="Compliance Finding" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1" count="1">
-        <m/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="Enforcement Action" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
-    </cacheField>
-    <cacheField name="Enforcement Status" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
-    </cacheField>
-    <cacheField name="Enforcement Document Number" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
-    </cacheField>
-    <cacheField name="Condition Number" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
-    </cacheField>
-    <cacheField name="Requirement Source" numFmtId="0">
       <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
     </cacheField>
     <cacheField name="IR Issuance Date" numFmtId="0">
@@ -607,101 +615,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{F3646FCF-C206-4361-8690-240132D1671E}" name="PivotTable24" cacheId="1018" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="K4:M9" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
-  <pivotFields count="13">
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="2">
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" dataField="1" showAll="0">
-      <items count="2">
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField axis="axisCol" showAll="0">
-      <items count="2">
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="2">
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="3">
-    <field x="2"/>
-    <field x="4"/>
-    <field x="6"/>
-  </rowFields>
-  <rowItems count="4">
-    <i>
-      <x/>
-    </i>
-    <i r="1">
-      <x/>
-    </i>
-    <i r="2">
-      <x/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colFields count="1">
-    <field x="5"/>
-  </colFields>
-  <colItems count="2">
-    <i>
-      <x/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Count of Enforcement Action" fld="4" subtotal="count" baseField="0" baseItem="0"/>
-  </dataFields>
-  <formats count="3">
-    <format dxfId="7">
-      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="8">
-      <pivotArea field="5" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
-    </format>
-    <format dxfId="9">
-      <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
-    </format>
-  </formats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{3A2CB471-5EA6-4127-A467-E8F5D9596452}" name="PivotTable23" cacheId="1024" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{3A2CB471-5EA6-4127-A467-E8F5D9596452}" name="PivotTable23" cacheId="1510" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="E4:G8" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="16">
     <pivotField showAll="0"/>
@@ -766,15 +680,6 @@
     <dataField name="Count of Summary" fld="2" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="6">
-    <format dxfId="1">
-      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="2">
-      <pivotArea field="6" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
-    </format>
-    <format dxfId="3">
-      <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
-    </format>
     <format dxfId="4">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
@@ -782,6 +687,15 @@
       <pivotArea field="6" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
     <format dxfId="6">
+      <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="7">
+      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="8">
+      <pivotArea field="6" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
+    </format>
+    <format dxfId="9">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -797,8 +711,8 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{DE23F307-6508-443D-9D35-8D0EAB9E4958}" name="PivotTable22" cacheId="1011" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{DE23F307-6508-443D-9D35-8D0EAB9E4958}" name="PivotTable22" cacheId="1522" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="B4:C6" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="8">
     <pivotField dataField="1" showAll="0"/>
@@ -844,6 +758,109 @@
 </pivotTableDefinition>
 </file>
 
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{F3646FCF-C206-4361-8690-240132D1671E}" name="PivotTable24" cacheId="1518" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="L6:N11" firstHeaderRow="1" firstDataRow="2" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
+  <pivotFields count="14">
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="2">
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisPage" showAll="0">
+      <items count="2">
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisRow" dataField="1" showAll="0">
+      <items count="2">
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisCol" showAll="0">
+      <items count="2">
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="2">
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="3">
+    <field x="2"/>
+    <field x="5"/>
+    <field x="7"/>
+  </rowFields>
+  <rowItems count="4">
+    <i>
+      <x/>
+    </i>
+    <i r="1">
+      <x/>
+    </i>
+    <i r="2">
+      <x/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="6"/>
+  </colFields>
+  <colItems count="2">
+    <i>
+      <x/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </colItems>
+  <pageFields count="1">
+    <pageField fld="4" hier="-1"/>
+  </pageFields>
+  <dataFields count="1">
+    <dataField name="Count of Enforcement Action" fld="5" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <formats count="3">
+    <format dxfId="1">
+      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="2">
+      <pivotArea field="6" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
+    </format>
+    <format dxfId="3">
+      <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+    </format>
+  </formats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{25A5AAF5-465E-40DA-80D8-7D63F24C71CF}" name="Inspections" displayName="Inspections" ref="A1:H2" totalsRowShown="0">
   <autoFilter ref="A1:H2" xr:uid="{25A5AAF5-465E-40DA-80D8-7D63F24C71CF}"/>
@@ -887,13 +904,14 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{BB558FF6-8E88-4B8C-85F0-A9AC1F3494E1}" name="Enforcements" displayName="Enforcements" ref="A1:M2" totalsRowShown="0">
-  <autoFilter ref="A1:M2" xr:uid="{BB558FF6-8E88-4B8C-85F0-A9AC1F3494E1}"/>
-  <tableColumns count="13">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{BB558FF6-8E88-4B8C-85F0-A9AC1F3494E1}" name="Enforcements" displayName="Enforcements" ref="A1:N2" totalsRowShown="0">
+  <autoFilter ref="A1:N2" xr:uid="{BB558FF6-8E88-4B8C-85F0-A9AC1F3494E1}"/>
+  <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{002DF4D9-2342-465C-AFA9-D19EC440D92D}" name="IR Number"/>
     <tableColumn id="2" xr3:uid="{121E0AA8-E00F-4A87-B2E8-39B632F930A5}" name="IR Progress"/>
     <tableColumn id="3" xr3:uid="{6A40920A-25DB-4945-B49C-37E79325503F}" name="Project Name"/>
     <tableColumn id="4" xr3:uid="{BFB4DB6B-0FE0-47F2-B2D1-38090A00D902}" name="Project Type"/>
+    <tableColumn id="14" xr3:uid="{0C33F754-7EED-4DC1-A065-4630AFD7D772}" name="Compliance Finding"/>
     <tableColumn id="5" xr3:uid="{EB406C39-C322-4377-9490-1E84DC84279E}" name="Enforcement Action"/>
     <tableColumn id="6" xr3:uid="{5C25DE55-141D-4A51-AF8A-3E0C7590A8B3}" name="Enforcement Status"/>
     <tableColumn id="7" xr3:uid="{6D85C97C-DB2A-45AC-8D60-9844F03DFAE0}" name="Enforcement Document Number"/>
@@ -1331,7 +1349,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FBAE1F1F-8658-4E77-804F-851BEEBDB0CE}">
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:N1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="2" width="14.5703125" customWidth="1"/>
@@ -1348,7 +1366,7 @@
     <col min="13" max="13" width="13.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13">
+    <row r="1" spans="1:14">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1362,30 +1380,33 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F1" t="s">
         <v>11</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>12</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>13</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>4</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>5</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>6</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>7</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>16</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>17</v>
       </c>
     </row>
@@ -1399,22 +1420,22 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C3DA8C2-D460-3E49-93A1-0DC80ABEB419}">
-  <dimension ref="B2:M33"/>
+  <dimension ref="B2:N33"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="14.28515625" customWidth="1"/>
     <col min="3" max="3" width="19.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12.140625" customWidth="1"/>
-    <col min="5" max="5" width="20.140625" customWidth="1"/>
+    <col min="5" max="5" width="18" customWidth="1"/>
     <col min="6" max="6" width="17.28515625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="11.7109375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="12" customWidth="1"/>
     <col min="9" max="9" width="27.5703125" customWidth="1"/>
     <col min="10" max="10" width="17.28515625" customWidth="1"/>
-    <col min="11" max="11" width="31.85546875" customWidth="1"/>
-    <col min="12" max="12" width="24" customWidth="1"/>
+    <col min="11" max="11" width="11.7109375" customWidth="1"/>
+    <col min="12" max="12" width="27.5703125" customWidth="1"/>
     <col min="13" max="13" width="17.28515625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="14" customWidth="1"/>
+    <col min="14" max="14" width="11.7109375" customWidth="1"/>
     <col min="15" max="15" width="13.140625" customWidth="1"/>
     <col min="16" max="16" width="15.7109375" customWidth="1"/>
     <col min="17" max="17" width="15.140625" customWidth="1"/>
@@ -1485,18 +1506,18 @@
     <col min="125" max="125" width="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:13">
+    <row r="2" spans="2:14">
       <c r="B2" t="s">
         <v>18</v>
       </c>
       <c r="E2" t="s">
         <v>19</v>
       </c>
-      <c r="K2" t="s">
+      <c r="L2" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="2:13">
+    <row r="4" spans="2:14">
       <c r="B4" s="1" t="s">
         <v>21</v>
       </c>
@@ -1510,15 +1531,14 @@
         <v>24</v>
       </c>
       <c r="G4" s="4"/>
-      <c r="K4" s="4" t="s">
+      <c r="L4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="M4" t="s">
         <v>25</v>
       </c>
-      <c r="L4" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="M4" s="4"/>
     </row>
-    <row r="5" spans="2:13">
+    <row r="5" spans="2:14">
       <c r="B5" s="2" t="s">
         <v>26</v>
       </c>
@@ -1532,17 +1552,8 @@
       <c r="G5" t="s">
         <v>27</v>
       </c>
-      <c r="K5" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="L5" t="s">
-        <v>26</v>
-      </c>
-      <c r="M5" t="s">
-        <v>27</v>
-      </c>
     </row>
-    <row r="6" spans="2:13">
+    <row r="6" spans="2:14">
       <c r="B6" s="2" t="s">
         <v>27</v>
       </c>
@@ -1552,42 +1563,62 @@
       </c>
       <c r="F6" s="6"/>
       <c r="G6" s="6"/>
-      <c r="K6" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="L6" s="6"/>
-      <c r="M6" s="6"/>
+      <c r="L6" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="M6" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="N6" s="4"/>
     </row>
-    <row r="7" spans="2:13">
+    <row r="7" spans="2:14">
       <c r="E7" s="3" t="s">
         <v>26</v>
       </c>
       <c r="F7" s="6"/>
       <c r="G7" s="6"/>
-      <c r="K7" s="3" t="s">
+      <c r="L7" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="M7" t="s">
         <v>26</v>
       </c>
-      <c r="L7" s="6"/>
-      <c r="M7" s="6"/>
+      <c r="N7" t="s">
+        <v>27</v>
+      </c>
     </row>
-    <row r="8" spans="2:13">
+    <row r="8" spans="2:14">
       <c r="E8" s="2" t="s">
         <v>27</v>
       </c>
       <c r="F8" s="6"/>
       <c r="G8" s="6"/>
-      <c r="K8" s="5" t="s">
+      <c r="L8" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="L8" s="6"/>
       <c r="M8" s="6"/>
+      <c r="N8" s="6"/>
     </row>
-    <row r="9" spans="2:13">
-      <c r="K9" s="2" t="s">
+    <row r="9" spans="2:14">
+      <c r="L9" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="M9" s="6"/>
+      <c r="N9" s="6"/>
+    </row>
+    <row r="10" spans="2:14">
+      <c r="L10" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="M10" s="6"/>
+      <c r="N10" s="6"/>
+    </row>
+    <row r="11" spans="2:14">
+      <c r="L11" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="L9" s="6"/>
-      <c r="M9" s="6"/>
+      <c r="M11" s="6"/>
+      <c r="N11" s="6"/>
     </row>
     <row r="33" spans="12:12"/>
   </sheetData>

</xml_diff>

<commit_message>
[Comp-751] CEB report excel tweaks
</commit_message>
<xml_diff>
--- a/compliance-api/src/compliance_api/services/report/ceb_template.xlsx
+++ b/compliance-api/src/compliance_api/services/report/ceb_template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30015"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30023"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tayalee/Desktop/Excel pivot tables_forfeedback/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="230" documentId="13_ncr:1_{0AC415D9-D733-894D-B4A0-A67D0E09A217}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9698F4B5-39DB-4005-8176-674D149EF680}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F8F9D94A-C55D-461C-B55F-659C33E62162}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="35080" yWindow="1540" windowWidth="34560" windowHeight="20260" firstSheet="3" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,9 +20,9 @@
   </sheets>
   <calcPr calcId="191028"/>
   <pivotCaches>
-    <pivotCache cacheId="1510" r:id="rId5"/>
-    <pivotCache cacheId="1518" r:id="rId6"/>
-    <pivotCache cacheId="1522" r:id="rId7"/>
+    <pivotCache cacheId="909" r:id="rId5"/>
+    <pivotCache cacheId="917" r:id="rId6"/>
+    <pivotCache cacheId="923" r:id="rId7"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -41,126 +41,6 @@
     </ext>
   </extLst>
 </workbook>
-</file>
-
-<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
-  <authors>
-    <author>Taya Lee</author>
-    <author>tc={077DFB58-63D9-8146-93DC-66E3FA1A6510}</author>
-  </authors>
-  <commentList>
-    <comment ref="B2" authorId="0" shapeId="0" xr:uid="{68C87A6D-DCE5-2B4E-BA31-D467C4C1DFA5}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="10"/>
-            <color rgb="FF000000"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Taya Lee:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <color rgb="FF000000"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <color rgb="FF000000"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Source = Inspections
-</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="E2" authorId="0" shapeId="0" xr:uid="{C154DB07-CF68-CC45-A7E6-EEC672264C41}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="10"/>
-            <color rgb="FF000000"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Taya Lee:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <color rgb="FF000000"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <color rgb="FF000000"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Source = Requirements</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="L2" authorId="0" shapeId="0" xr:uid="{54A4951F-359C-2B4C-B5F0-8D56596EFF78}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="10"/>
-            <color rgb="FF000000"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Taya Lee:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <color rgb="FF000000"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <color rgb="FF000000"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Source = Enforcements
-</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="L33" authorId="1" shapeId="0" xr:uid="{077DFB58-63D9-8146-93DC-66E3FA1A6510}">
-      <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-    This example shows how this Order is accounted for 10 times in the table, because it was one Order for 10 Requirements</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
 </file>
 
 <file path=xl/connections.xml><?xml version="1.0" encoding="utf-8"?>
@@ -280,26 +160,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -431,58 +298,24 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <person displayName="Lee, Taya EAO:EX" id="{58657C1B-1CA6-314F-B79D-36CCFB346E28}" userId="S::Taya.Lee@gov.bc.ca::b8076c1d-e35e-402e-9405-dceb8aeb9fb9" providerId="AD"/>
-</personList>
-</file>
-
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshOnLoad="1" refreshedBy="Excel Services" refreshedDate="46134.432263078706" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="1" xr:uid="{E508D2FB-1B6C-4B04-92EF-07C92A3B7FD7}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshOnLoad="1" refreshedBy="Excel Services" refreshedDate="46142.683587847219" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="1" xr:uid="{9A655F1F-804E-4F57-A400-987732F35DAD}">
   <cacheSource type="worksheet">
-    <worksheetSource name="Requirements"/>
+    <worksheetSource name="Inspections"/>
   </cacheSource>
-  <cacheFields count="16">
+  <cacheFields count="8">
     <cacheField name="IR Number" numFmtId="0">
       <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
     </cacheField>
-    <cacheField name="Topic" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
-    </cacheField>
-    <cacheField name="Summary" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
-    </cacheField>
     <cacheField name="IR Progress" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
-    </cacheField>
-    <cacheField name="Project Name" numFmtId="0">
       <sharedItems containsNonDate="0" containsString="0" containsBlank="1" count="1">
         <m/>
       </sharedItems>
     </cacheField>
+    <cacheField name="Project Name" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
     <cacheField name="Project Type" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1" count="1">
-        <m/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="Compliance Finding" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1" count="1">
-        <m/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="Enforcement Action" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
-    </cacheField>
-    <cacheField name="Enforcement Status" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
-    </cacheField>
-    <cacheField name="Enforcement Document Number" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
-    </cacheField>
-    <cacheField name="Condition Number" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
-    </cacheField>
-    <cacheField name="Requirement Source" numFmtId="0">
       <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
     </cacheField>
     <cacheField name="IR Issuance Date" numFmtId="0">
@@ -507,7 +340,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshOnLoad="1" refreshedBy="Excel Services" refreshedDate="46134.432263194445" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="1" xr:uid="{3DC42666-42A1-448D-A623-A82BC44CBAFC}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshOnLoad="1" refreshedBy="Excel Services" refreshedDate="46142.683587847219" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="1" xr:uid="{3DC42666-42A1-448D-A623-A82BC44CBAFC}">
   <cacheSource type="worksheet">
     <worksheetSource name="Enforcements"/>
   </cacheSource>
@@ -574,23 +407,51 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshOnLoad="1" refreshedBy="Excel Services" refreshedDate="46134.432263194445" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="1" xr:uid="{9A655F1F-804E-4F57-A400-987732F35DAD}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshOnLoad="1" refreshedBy="Excel Services" refreshedDate="46142.683587847219" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="1" xr:uid="{E508D2FB-1B6C-4B04-92EF-07C92A3B7FD7}">
   <cacheSource type="worksheet">
-    <worksheetSource name="Inspections"/>
+    <worksheetSource name="Requirements"/>
   </cacheSource>
-  <cacheFields count="8">
+  <cacheFields count="16">
     <cacheField name="IR Number" numFmtId="0">
       <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
     </cacheField>
+    <cacheField name="Topic" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="Summary" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
     <cacheField name="IR Progress" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="Project Name" numFmtId="0">
       <sharedItems containsNonDate="0" containsString="0" containsBlank="1" count="1">
         <m/>
       </sharedItems>
     </cacheField>
-    <cacheField name="Project Name" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
-    </cacheField>
     <cacheField name="Project Type" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1" count="1">
+        <m/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Compliance Finding" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1" count="1">
+        <m/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Enforcement Action" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="Enforcement Status" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="Enforcement Document Number" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="Condition Number" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="Requirement Source" numFmtId="0">
       <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
     </cacheField>
     <cacheField name="IR Issuance Date" numFmtId="0">
@@ -615,7 +476,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{3A2CB471-5EA6-4127-A467-E8F5D9596452}" name="PivotTable23" cacheId="1510" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{3A2CB471-5EA6-4127-A467-E8F5D9596452}" name="PivotTable23" cacheId="923" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="E4:G8" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="16">
     <pivotField showAll="0"/>
@@ -712,7 +573,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{DE23F307-6508-443D-9D35-8D0EAB9E4958}" name="PivotTable22" cacheId="1522" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{DE23F307-6508-443D-9D35-8D0EAB9E4958}" name="PivotTable22" cacheId="909" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="B4:C6" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="8">
     <pivotField dataField="1" showAll="0"/>
@@ -759,8 +620,8 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{F3646FCF-C206-4361-8690-240132D1671E}" name="PivotTable24" cacheId="1518" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="L6:N11" firstHeaderRow="1" firstDataRow="2" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{F3646FCF-C206-4361-8690-240132D1671E}" name="PivotTable24" cacheId="917" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="K6:M11" firstHeaderRow="1" firstDataRow="2" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="14">
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
@@ -1209,14 +1070,6 @@
 </a:theme>
 </file>
 
-<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
-<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="L33" dT="2026-03-18T17:17:25.75" personId="{58657C1B-1CA6-314F-B79D-36CCFB346E28}" id="{077DFB58-63D9-8146-93DC-66E3FA1A6510}">
-    <text>This example shows how this Order is accounted for 10 times in the table, because it was one Order for 10 Requirements</text>
-  </threadedComment>
-</ThreadedComments>
-</file>
-
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C91F6D2A-2426-4151-8DB7-092E919C69C7}">
   <dimension ref="A1:H1"/>
@@ -1419,8 +1272,8 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C3DA8C2-D460-3E49-93A1-0DC80ABEB419}">
-  <dimension ref="B2:N33"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C3DA8C2-D460-3E49-93A1-0DC80ABEB419}">
+  <dimension ref="B2:M11"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="14.28515625" customWidth="1"/>
@@ -1432,92 +1285,91 @@
     <col min="8" max="8" width="12" customWidth="1"/>
     <col min="9" max="9" width="27.5703125" customWidth="1"/>
     <col min="10" max="10" width="17.28515625" customWidth="1"/>
-    <col min="11" max="11" width="11.7109375" customWidth="1"/>
-    <col min="12" max="12" width="27.5703125" customWidth="1"/>
-    <col min="13" max="13" width="17.28515625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11.7109375" customWidth="1"/>
-    <col min="15" max="15" width="13.140625" customWidth="1"/>
-    <col min="16" max="16" width="15.7109375" customWidth="1"/>
-    <col min="17" max="17" width="15.140625" customWidth="1"/>
-    <col min="18" max="18" width="12.28515625" customWidth="1"/>
-    <col min="19" max="19" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="7.42578125" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="24.42578125" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="24.42578125" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="24.42578125" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="24.42578125" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="20.140625" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="29" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="22.42578125" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="23" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="22.42578125" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="37" max="41" width="23.140625" bestFit="1" customWidth="1"/>
-    <col min="42" max="43" width="23.42578125" bestFit="1" customWidth="1"/>
-    <col min="44" max="45" width="24.42578125" bestFit="1" customWidth="1"/>
-    <col min="46" max="47" width="24.140625" bestFit="1" customWidth="1"/>
-    <col min="48" max="48" width="22.85546875" bestFit="1" customWidth="1"/>
-    <col min="49" max="50" width="23.7109375" bestFit="1" customWidth="1"/>
-    <col min="51" max="51" width="23.28515625" bestFit="1" customWidth="1"/>
-    <col min="52" max="53" width="22.42578125" bestFit="1" customWidth="1"/>
-    <col min="54" max="56" width="23.140625" bestFit="1" customWidth="1"/>
-    <col min="57" max="57" width="24.140625" bestFit="1" customWidth="1"/>
-    <col min="58" max="58" width="23.7109375" bestFit="1" customWidth="1"/>
-    <col min="59" max="61" width="24.140625" bestFit="1" customWidth="1"/>
-    <col min="62" max="62" width="25.140625" bestFit="1" customWidth="1"/>
-    <col min="63" max="63" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="64" max="64" width="37.7109375" bestFit="1" customWidth="1"/>
-    <col min="65" max="65" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="66" max="66" width="22.42578125" bestFit="1" customWidth="1"/>
-    <col min="67" max="67" width="27.42578125" bestFit="1" customWidth="1"/>
-    <col min="68" max="69" width="22.85546875" bestFit="1" customWidth="1"/>
-    <col min="70" max="73" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="74" max="74" width="11" bestFit="1" customWidth="1"/>
-    <col min="75" max="83" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="84" max="84" width="23" bestFit="1" customWidth="1"/>
-    <col min="85" max="85" width="22.7109375" bestFit="1" customWidth="1"/>
-    <col min="86" max="86" width="22.140625" bestFit="1" customWidth="1"/>
-    <col min="87" max="87" width="21.7109375" bestFit="1" customWidth="1"/>
-    <col min="88" max="89" width="20.85546875" bestFit="1" customWidth="1"/>
-    <col min="90" max="92" width="22.42578125" bestFit="1" customWidth="1"/>
-    <col min="93" max="94" width="23.42578125" bestFit="1" customWidth="1"/>
-    <col min="95" max="95" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="96" max="98" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="99" max="100" width="4.28515625" bestFit="1" customWidth="1"/>
-    <col min="101" max="101" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="102" max="102" width="15" bestFit="1" customWidth="1"/>
-    <col min="103" max="103" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="104" max="114" width="22.85546875" bestFit="1" customWidth="1"/>
-    <col min="115" max="116" width="11" bestFit="1" customWidth="1"/>
-    <col min="117" max="117" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="118" max="118" width="22.140625" bestFit="1" customWidth="1"/>
-    <col min="119" max="119" width="22.85546875" bestFit="1" customWidth="1"/>
-    <col min="120" max="120" width="22.140625" bestFit="1" customWidth="1"/>
-    <col min="121" max="121" width="21" bestFit="1" customWidth="1"/>
-    <col min="122" max="122" width="17.42578125" bestFit="1" customWidth="1"/>
-    <col min="123" max="123" width="8" bestFit="1" customWidth="1"/>
-    <col min="124" max="124" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="125" max="125" width="10" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="27.5703125" customWidth="1"/>
+    <col min="12" max="12" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.7109375" customWidth="1"/>
+    <col min="14" max="14" width="13.140625" customWidth="1"/>
+    <col min="15" max="15" width="15.7109375" customWidth="1"/>
+    <col min="16" max="16" width="15.140625" customWidth="1"/>
+    <col min="17" max="17" width="12.28515625" customWidth="1"/>
+    <col min="18" max="18" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="7.42578125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="24.42578125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="24.42578125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="24.42578125" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="24.42578125" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="20.140625" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="29" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="22.42578125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="23" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="22.42578125" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="36" max="40" width="23.140625" bestFit="1" customWidth="1"/>
+    <col min="41" max="42" width="23.42578125" bestFit="1" customWidth="1"/>
+    <col min="43" max="44" width="24.42578125" bestFit="1" customWidth="1"/>
+    <col min="45" max="46" width="24.140625" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="22.85546875" bestFit="1" customWidth="1"/>
+    <col min="48" max="49" width="23.7109375" bestFit="1" customWidth="1"/>
+    <col min="50" max="50" width="23.28515625" bestFit="1" customWidth="1"/>
+    <col min="51" max="52" width="22.42578125" bestFit="1" customWidth="1"/>
+    <col min="53" max="55" width="23.140625" bestFit="1" customWidth="1"/>
+    <col min="56" max="56" width="24.140625" bestFit="1" customWidth="1"/>
+    <col min="57" max="57" width="23.7109375" bestFit="1" customWidth="1"/>
+    <col min="58" max="60" width="24.140625" bestFit="1" customWidth="1"/>
+    <col min="61" max="61" width="25.140625" bestFit="1" customWidth="1"/>
+    <col min="62" max="62" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="63" max="63" width="37.7109375" bestFit="1" customWidth="1"/>
+    <col min="64" max="64" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="65" max="65" width="22.42578125" bestFit="1" customWidth="1"/>
+    <col min="66" max="66" width="27.42578125" bestFit="1" customWidth="1"/>
+    <col min="67" max="68" width="22.85546875" bestFit="1" customWidth="1"/>
+    <col min="69" max="72" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="73" max="73" width="11" bestFit="1" customWidth="1"/>
+    <col min="74" max="82" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="83" max="83" width="23" bestFit="1" customWidth="1"/>
+    <col min="84" max="84" width="22.7109375" bestFit="1" customWidth="1"/>
+    <col min="85" max="85" width="22.140625" bestFit="1" customWidth="1"/>
+    <col min="86" max="86" width="21.7109375" bestFit="1" customWidth="1"/>
+    <col min="87" max="88" width="20.85546875" bestFit="1" customWidth="1"/>
+    <col min="89" max="91" width="22.42578125" bestFit="1" customWidth="1"/>
+    <col min="92" max="93" width="23.42578125" bestFit="1" customWidth="1"/>
+    <col min="94" max="94" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="95" max="97" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="98" max="99" width="4.28515625" bestFit="1" customWidth="1"/>
+    <col min="100" max="100" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="101" max="101" width="15" bestFit="1" customWidth="1"/>
+    <col min="102" max="102" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="103" max="113" width="22.85546875" bestFit="1" customWidth="1"/>
+    <col min="114" max="115" width="11" bestFit="1" customWidth="1"/>
+    <col min="116" max="116" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="117" max="117" width="22.140625" bestFit="1" customWidth="1"/>
+    <col min="118" max="118" width="22.85546875" bestFit="1" customWidth="1"/>
+    <col min="119" max="119" width="22.140625" bestFit="1" customWidth="1"/>
+    <col min="120" max="120" width="21" bestFit="1" customWidth="1"/>
+    <col min="121" max="121" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="122" max="122" width="8" bestFit="1" customWidth="1"/>
+    <col min="123" max="123" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="124" max="124" width="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:14">
+    <row r="2" spans="2:13">
       <c r="B2" t="s">
         <v>18</v>
       </c>
       <c r="E2" t="s">
         <v>19</v>
       </c>
-      <c r="L2" t="s">
+      <c r="K2" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="2:14">
+    <row r="4" spans="2:13">
       <c r="B4" s="1" t="s">
         <v>21</v>
       </c>
@@ -1531,14 +1383,14 @@
         <v>24</v>
       </c>
       <c r="G4" s="4"/>
-      <c r="L4" s="1" t="s">
+      <c r="K4" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="M4" t="s">
+      <c r="L4" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="2:14">
+    <row r="5" spans="2:13">
       <c r="B5" s="2" t="s">
         <v>26</v>
       </c>
@@ -1553,7 +1405,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="6" spans="2:14">
+    <row r="6" spans="2:13">
       <c r="B6" s="2" t="s">
         <v>27</v>
       </c>
@@ -1563,67 +1415,65 @@
       </c>
       <c r="F6" s="6"/>
       <c r="G6" s="6"/>
+      <c r="K6" s="4" t="s">
+        <v>28</v>
+      </c>
       <c r="L6" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="M6" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="N6" s="4"/>
+      <c r="M6" s="4"/>
     </row>
-    <row r="7" spans="2:14">
+    <row r="7" spans="2:13">
       <c r="E7" s="3" t="s">
         <v>26</v>
       </c>
       <c r="F7" s="6"/>
       <c r="G7" s="6"/>
-      <c r="L7" s="1" t="s">
+      <c r="K7" s="1" t="s">
         <v>21</v>
       </c>
+      <c r="L7" t="s">
+        <v>26</v>
+      </c>
       <c r="M7" t="s">
-        <v>26</v>
-      </c>
-      <c r="N7" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="8" spans="2:14">
+    <row r="8" spans="2:13">
       <c r="E8" s="2" t="s">
         <v>27</v>
       </c>
       <c r="F8" s="6"/>
       <c r="G8" s="6"/>
-      <c r="L8" s="2" t="s">
+      <c r="K8" s="2" t="s">
         <v>26</v>
       </c>
+      <c r="L8" s="6"/>
       <c r="M8" s="6"/>
-      <c r="N8" s="6"/>
     </row>
-    <row r="9" spans="2:14">
-      <c r="L9" s="3" t="s">
+    <row r="9" spans="2:13">
+      <c r="K9" s="3" t="s">
         <v>26</v>
       </c>
+      <c r="L9" s="6"/>
       <c r="M9" s="6"/>
-      <c r="N9" s="6"/>
     </row>
-    <row r="10" spans="2:14">
-      <c r="L10" s="5" t="s">
+    <row r="10" spans="2:13">
+      <c r="K10" s="5" t="s">
         <v>26</v>
       </c>
+      <c r="L10" s="6"/>
       <c r="M10" s="6"/>
-      <c r="N10" s="6"/>
     </row>
-    <row r="11" spans="2:14">
-      <c r="L11" s="2" t="s">
+    <row r="11" spans="2:13">
+      <c r="K11" s="2" t="s">
         <v>27</v>
       </c>
+      <c r="L11" s="6"/>
       <c r="M11" s="6"/>
-      <c r="N11" s="6"/>
     </row>
-    <row r="33" spans="12:12"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing r:id="rId4"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
[Comp-751-2] CEB Summary report add complaints and pivot tables
</commit_message>
<xml_diff>
--- a/compliance-api/src/compliance_api/services/report/ceb_template.xlsx
+++ b/compliance-api/src/compliance_api/services/report/ceb_template.xlsx
@@ -2,27 +2,30 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30023"/>
-  <workbookPr/>
+  <workbookPr hidePivotFieldList="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tayalee/Desktop/Excel pivot tables_forfeedback/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F8F9D94A-C55D-461C-B55F-659C33E62162}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{006F340F-4539-428D-9C2A-553C09694AAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="35080" yWindow="1540" windowWidth="34560" windowHeight="20260" firstSheet="3" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Inspections" sheetId="13" r:id="rId1"/>
     <sheet name="Requirements" sheetId="11" r:id="rId2"/>
-    <sheet name="Enforcements" sheetId="12" r:id="rId3"/>
-    <sheet name="Insights" sheetId="3" r:id="rId4"/>
+    <sheet name="Enforcement" sheetId="12" r:id="rId3"/>
+    <sheet name="InsightsInsights" sheetId="3" r:id="rId4"/>
+    <sheet name="Complaints" sheetId="14" r:id="rId5"/>
+    <sheet name="ComplaintsInsights" sheetId="15" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191028"/>
   <pivotCaches>
-    <pivotCache cacheId="909" r:id="rId5"/>
-    <pivotCache cacheId="917" r:id="rId6"/>
-    <pivotCache cacheId="923" r:id="rId7"/>
+    <pivotCache cacheId="501" r:id="rId7"/>
+    <pivotCache cacheId="509" r:id="rId8"/>
+    <pivotCache cacheId="515" r:id="rId9"/>
+    <pivotCache cacheId="525" r:id="rId10"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -41,6 +44,31 @@
     </ext>
   </extLst>
 </workbook>
+</file>
+
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>Tolk, Shaelyn EAO:EX</author>
+  </authors>
+  <commentList>
+    <comment ref="B2" authorId="0" shapeId="0" xr:uid="{83AAB37E-1AAA-4CC9-A0B6-FE8C22AF5EDF}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t xml:space="preserve">Inspections that have been Canceled or Closed as note to file will not appear in the Inspection Records totals.
+</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/connections.xml><?xml version="1.0" encoding="utf-8"?>
@@ -67,7 +95,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="41">
   <si>
     <t>IR Number</t>
   </si>
@@ -123,13 +151,13 @@
     <t>Unique Key</t>
   </si>
   <si>
-    <t>Number of Inspections</t>
-  </si>
-  <si>
-    <t>Inspection Requirements Distribution by Project/Type</t>
-  </si>
-  <si>
-    <t>Enforcement Distribution</t>
+    <t>Inspection Records</t>
+  </si>
+  <si>
+    <t>Compliance Findings by Sector and Project</t>
+  </si>
+  <si>
+    <t>Enforcement Summary by Project</t>
   </si>
   <si>
     <t>Row Labels</t>
@@ -154,19 +182,62 @@
   </si>
   <si>
     <t>Count of Enforcement Action</t>
+  </si>
+  <si>
+    <t>Complaint Number</t>
+  </si>
+  <si>
+    <t>Date Received</t>
+  </si>
+  <si>
+    <t>Complaint Source</t>
+  </si>
+  <si>
+    <t>Complaint Source Details</t>
+  </si>
+  <si>
+    <t>Complaint Status</t>
+  </si>
+  <si>
+    <t>Complaint Resolution</t>
+  </si>
+  <si>
+    <t>Complaint Source and Resolution Summary</t>
+  </si>
+  <si>
+    <t>Complaint Sources by Project</t>
+  </si>
+  <si>
+    <t>Project Complaints by Topic and Resolution</t>
+  </si>
+  <si>
+    <t>Count of Complaint Number</t>
+  </si>
+  <si>
+    <t>Count of Complaint Source</t>
+  </si>
+  <si>
+    <t>Count of Complaint Resolution</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -183,7 +254,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -191,11 +262,26 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -208,18 +294,121 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" indent="2"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="10">
+  <dxfs count="25">
     <dxf>
       <fill>
         <patternFill patternType="none">
           <fgColor indexed="64"/>
           <bgColor indexed="65"/>
         </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.39997558519241921"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.39997558519241921"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.39997558519241921"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.39997558519241921"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.39997558519241921"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.39997558519241921"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none"/>
       </fill>
     </dxf>
     <dxf>
@@ -299,7 +488,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshOnLoad="1" refreshedBy="Excel Services" refreshedDate="46142.683587847219" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="1" xr:uid="{9A655F1F-804E-4F57-A400-987732F35DAD}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshOnLoad="1" refreshedBy="Excel Services" refreshedDate="46148.598844328706" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="1" xr:uid="{9A655F1F-804E-4F57-A400-987732F35DAD}">
   <cacheSource type="worksheet">
     <worksheetSource name="Inspections"/>
   </cacheSource>
@@ -340,9 +529,9 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshOnLoad="1" refreshedBy="Excel Services" refreshedDate="46142.683587847219" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="1" xr:uid="{3DC42666-42A1-448D-A623-A82BC44CBAFC}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshOnLoad="1" refreshedBy="Excel Services" refreshedDate="46148.598844328706" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="1" xr:uid="{3DC42666-42A1-448D-A623-A82BC44CBAFC}">
   <cacheSource type="worksheet">
-    <worksheetSource name="Enforcements"/>
+    <worksheetSource name="Enforcement"/>
   </cacheSource>
   <cacheFields count="14">
     <cacheField name="IR Number" numFmtId="0">
@@ -407,7 +596,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshOnLoad="1" refreshedBy="Excel Services" refreshedDate="46142.683587847219" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="1" xr:uid="{E508D2FB-1B6C-4B04-92EF-07C92A3B7FD7}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshOnLoad="1" refreshedBy="Excel Services" refreshedDate="46148.598844328706" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="1" xr:uid="{E508D2FB-1B6C-4B04-92EF-07C92A3B7FD7}">
   <cacheSource type="worksheet">
     <worksheetSource name="Requirements"/>
   </cacheSource>
@@ -475,9 +664,71 @@
 </pivotCacheDefinition>
 </file>
 
+<file path=xl/pivotCache/pivotCacheDefinition4.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshOnLoad="1" refreshedBy="Excel Services" refreshedDate="46148.598844328706" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="1" xr:uid="{489B308B-C5F1-4496-9EA3-999C745CB76D}">
+  <cacheSource type="worksheet">
+    <worksheetSource name="Complaints"/>
+  </cacheSource>
+  <cacheFields count="11">
+    <cacheField name="Complaint Number" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1" count="1">
+        <m/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Project Name" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1" count="1">
+        <m/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Project Type" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1" count="1">
+        <m/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Topic" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1" count="1">
+        <m/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Date Received" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="Complaint Source" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1" count="1">
+        <m/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Complaint Source Details" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1" count="1">
+        <m/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Primary Officer" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="Complaint Status" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="Complaint Resolution" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1" count="1">
+        <m/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Case File Number" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+  </cacheFields>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
+      <x14:pivotCacheDefinition/>
+    </ext>
+  </extLst>
+</pivotCacheDefinition>
+</file>
+
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{3A2CB471-5EA6-4127-A467-E8F5D9596452}" name="PivotTable23" cacheId="923" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="E4:G8" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{3A2CB471-5EA6-4127-A467-E8F5D9596452}" name="PivotTable23" cacheId="515" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="E4:G7" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="16">
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
@@ -491,7 +742,7 @@
     </pivotField>
     <pivotField axis="axisRow" showAll="0">
       <items count="2">
-        <item x="0"/>
+        <item sd="0" x="0"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -515,11 +766,8 @@
     <field x="5"/>
     <field x="4"/>
   </rowFields>
-  <rowItems count="3">
+  <rowItems count="2">
     <i>
-      <x/>
-    </i>
-    <i r="1">
       <x/>
     </i>
     <i t="grand">
@@ -541,22 +789,22 @@
     <dataField name="Count of Summary" fld="2" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="6">
-    <format dxfId="4">
+    <format dxfId="19">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="5">
+    <format dxfId="20">
       <pivotArea field="6" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="6">
+    <format dxfId="21">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="7">
+    <format dxfId="22">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="8">
+    <format dxfId="23">
       <pivotArea field="6" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="9">
+    <format dxfId="24">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -573,7 +821,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{DE23F307-6508-443D-9D35-8D0EAB9E4958}" name="PivotTable22" cacheId="909" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{DE23F307-6508-443D-9D35-8D0EAB9E4958}" name="PivotTable22" cacheId="501" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="B4:C6" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="8">
     <pivotField dataField="1" showAll="0"/>
@@ -620,7 +868,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{F3646FCF-C206-4361-8690-240132D1671E}" name="PivotTable24" cacheId="917" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{F3646FCF-C206-4361-8690-240132D1671E}" name="PivotTable24" cacheId="509" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="K6:M11" firstHeaderRow="1" firstDataRow="2" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="14">
     <pivotField showAll="0"/>
@@ -700,13 +948,286 @@
     <dataField name="Count of Enforcement Action" fld="5" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="3">
+    <format dxfId="16">
+      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="17">
+      <pivotArea field="6" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
+    </format>
+    <format dxfId="18">
+      <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+    </format>
+  </formats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{49EF033C-CFA8-44B9-BC70-D0C253FFC2B0}" name="Project Complaints by Topic and Resolution" cacheId="525" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="Q4:S9" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="11">
+    <pivotField axis="axisRow" showAll="0">
+      <items count="2">
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="2">
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="2">
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisCol" dataField="1" showAll="0">
+      <items count="2">
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="3">
+    <field x="1"/>
+    <field x="3"/>
+    <field x="0"/>
+  </rowFields>
+  <rowItems count="4">
+    <i>
+      <x/>
+    </i>
+    <i r="1">
+      <x/>
+    </i>
+    <i r="2">
+      <x/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="9"/>
+  </colFields>
+  <colItems count="2">
+    <i>
+      <x/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Count of Complaint Resolution" fld="9" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <formats count="5">
+    <format dxfId="11">
+      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="12">
+      <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="13">
+      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="14">
+      <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="15">
+      <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+    </format>
+  </formats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{4DC00558-9D6A-4D8C-A8BC-4CABB5BCD879}" name="Complaint Sources by Project" cacheId="525" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="I4:K7" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="11">
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="2">
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="2">
+        <item sd="0" x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisCol" dataField="1" showAll="0">
+      <items count="2">
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="2">
+    <field x="2"/>
+    <field x="1"/>
+  </rowFields>
+  <rowItems count="2">
+    <i>
+      <x/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="5"/>
+  </colFields>
+  <colItems count="2">
+    <i>
+      <x/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Count of Complaint Source" fld="5" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <formats count="5">
+    <format dxfId="6">
+      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="7">
+      <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="8">
+      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="9">
+      <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="10">
+      <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+    </format>
+  </formats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{A78A3DE9-337B-4375-ABAF-39D54018E350}" name="Complaint Source and Resolution Summary" cacheId="525" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="B4:D8" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="11">
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="2">
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="2">
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisCol" showAll="0">
+      <items count="2">
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="2">
+    <field x="5"/>
+    <field x="6"/>
+  </rowFields>
+  <rowItems count="3">
+    <i>
+      <x/>
+    </i>
+    <i r="1">
+      <x/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="9"/>
+  </colFields>
+  <colItems count="2">
+    <i>
+      <x/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Count of Complaint Number" fld="0" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <formats count="5">
     <format dxfId="1">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
     <format dxfId="2">
-      <pivotArea field="6" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
+      <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
     <format dxfId="3">
+      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="4">
+      <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="5">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -765,7 +1286,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{BB558FF6-8E88-4B8C-85F0-A9AC1F3494E1}" name="Enforcements" displayName="Enforcements" ref="A1:N2" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{BB558FF6-8E88-4B8C-85F0-A9AC1F3494E1}" name="Enforcement" displayName="Enforcement" ref="A1:N2" totalsRowShown="0">
   <autoFilter ref="A1:N2" xr:uid="{BB558FF6-8E88-4B8C-85F0-A9AC1F3494E1}"/>
   <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{002DF4D9-2342-465C-AFA9-D19EC440D92D}" name="IR Number"/>
@@ -782,6 +1303,26 @@
     <tableColumn id="11" xr3:uid="{82D63C41-2FDB-4AE6-AE02-192508539839}" name="Case File Number"/>
     <tableColumn id="12" xr3:uid="{639BF936-83D9-4FBE-8CB2-DF921632AE61}" name="Index"/>
     <tableColumn id="13" xr3:uid="{7E13429B-9F97-48D0-BE0A-1E9CE9D0A7C0}" name="Unique Key"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{A87B5369-917C-4BBD-9D07-5706A9AED13B}" name="Complaints" displayName="Complaints" ref="A1:K2" insertRow="1" totalsRowShown="0">
+  <autoFilter ref="A1:K2" xr:uid="{A87B5369-917C-4BBD-9D07-5706A9AED13B}"/>
+  <tableColumns count="11">
+    <tableColumn id="1" xr3:uid="{227CB843-AAB1-4F7C-8E2A-DB61E33497D6}" name="Complaint Number"/>
+    <tableColumn id="3" xr3:uid="{93A4A499-0455-49F4-B4FB-BEC8221A720C}" name="Project Name"/>
+    <tableColumn id="4" xr3:uid="{D48FB694-ADCC-426D-993E-720B570F7600}" name="Project Type"/>
+    <tableColumn id="2" xr3:uid="{6D2553B0-FA95-49DC-A4E2-9D71506573DA}" name="Topic"/>
+    <tableColumn id="5" xr3:uid="{240065E5-AEA8-4991-B3F4-2E79B2412A1C}" name="Date Received"/>
+    <tableColumn id="6" xr3:uid="{0AA8DD19-931D-4EF5-B979-8FB501BD88A8}" name="Complaint Source"/>
+    <tableColumn id="7" xr3:uid="{093E4DD5-733F-4E21-BBCF-20E4089ED0DA}" name="Complaint Source Details"/>
+    <tableColumn id="8" xr3:uid="{27CD44B6-B993-42F6-9D05-8161443FB73A}" name="Primary Officer"/>
+    <tableColumn id="10" xr3:uid="{329A32BD-B57C-4124-87F8-80921AC20A9E}" name="Complaint Status"/>
+    <tableColumn id="9" xr3:uid="{C68E3C04-92F4-4069-80A6-464DAE5D9516}" name="Complaint Resolution"/>
+    <tableColumn id="11" xr3:uid="{74150121-EE4E-45AF-96A6-3452679C965A}" name="Case File Number"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1272,7 +1813,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C3DA8C2-D460-3E49-93A1-0DC80ABEB419}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C3DA8C2-D460-3E49-93A1-0DC80ABEB419}">
   <dimension ref="B2:M11"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
   <cols>
@@ -1282,7 +1823,7 @@
     <col min="5" max="5" width="18" customWidth="1"/>
     <col min="6" max="6" width="17.28515625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12" customWidth="1"/>
+    <col min="8" max="8" width="11.7109375" customWidth="1"/>
     <col min="9" max="9" width="27.5703125" customWidth="1"/>
     <col min="10" max="10" width="17.28515625" customWidth="1"/>
     <col min="11" max="11" width="27.5703125" customWidth="1"/>
@@ -1394,7 +1935,7 @@
       <c r="B5" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C5" s="6"/>
+      <c r="C5" s="7"/>
       <c r="E5" s="1" t="s">
         <v>21</v>
       </c>
@@ -1409,12 +1950,12 @@
       <c r="B6" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="C6" s="6"/>
+      <c r="C6" s="7"/>
       <c r="E6" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="F6" s="6"/>
-      <c r="G6" s="6"/>
+      <c r="F6" s="7"/>
+      <c r="G6" s="7"/>
       <c r="K6" s="4" t="s">
         <v>28</v>
       </c>
@@ -1424,11 +1965,11 @@
       <c r="M6" s="4"/>
     </row>
     <row r="7" spans="2:13">
-      <c r="E7" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="F7" s="6"/>
-      <c r="G7" s="6"/>
+      <c r="E7" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F7" s="7"/>
+      <c r="G7" s="7"/>
       <c r="K7" s="1" t="s">
         <v>21</v>
       </c>
@@ -1440,37 +1981,286 @@
       </c>
     </row>
     <row r="8" spans="2:13">
-      <c r="E8" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F8" s="6"/>
-      <c r="G8" s="6"/>
       <c r="K8" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="L8" s="6"/>
-      <c r="M8" s="6"/>
+      <c r="L8" s="7"/>
+      <c r="M8" s="7"/>
     </row>
     <row r="9" spans="2:13">
       <c r="K9" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="L9" s="6"/>
-      <c r="M9" s="6"/>
+      <c r="L9" s="7"/>
+      <c r="M9" s="7"/>
     </row>
     <row r="10" spans="2:13">
       <c r="K10" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="L10" s="6"/>
-      <c r="M10" s="6"/>
+      <c r="L10" s="7"/>
+      <c r="M10" s="7"/>
     </row>
     <row r="11" spans="2:13">
       <c r="K11" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="L11" s="6"/>
-      <c r="M11" s="6"/>
+      <c r="L11" s="7"/>
+      <c r="M11" s="7"/>
+    </row>
+  </sheetData>
+  <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0" pivotTables="0"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId4"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02D60FF9-2075-415C-B0EA-3DDAF185196F}">
+  <dimension ref="A1:K1"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="20.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="22.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="19.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11">
+      <c r="A1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F1" t="s">
+        <v>31</v>
+      </c>
+      <c r="G1" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1" t="s">
+        <v>5</v>
+      </c>
+      <c r="I1" t="s">
+        <v>33</v>
+      </c>
+      <c r="J1" t="s">
+        <v>34</v>
+      </c>
+      <c r="K1" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{668EBFF0-F7C1-4563-9C72-94D19E58850B}">
+  <dimension ref="B2:S24"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="2" max="2" width="26.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="25.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="29" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="11.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:19">
+      <c r="B2" t="s">
+        <v>35</v>
+      </c>
+      <c r="I2" t="s">
+        <v>36</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="4" spans="2:19">
+      <c r="B4" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D4" s="8"/>
+      <c r="I4" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="K4" s="8"/>
+      <c r="Q4" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="R4" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="S4" s="8"/>
+    </row>
+    <row r="5" spans="2:19">
+      <c r="B5" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D5" t="s">
+        <v>27</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="J5" t="s">
+        <v>26</v>
+      </c>
+      <c r="K5" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q5" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="R5" t="s">
+        <v>26</v>
+      </c>
+      <c r="S5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="6" spans="2:19">
+      <c r="B6" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C6" s="7"/>
+      <c r="D6" s="7"/>
+      <c r="I6" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="J6" s="7"/>
+      <c r="K6" s="7"/>
+      <c r="Q6" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="R6" s="7"/>
+      <c r="S6" s="7"/>
+    </row>
+    <row r="7" spans="2:19">
+      <c r="B7" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C7" s="7"/>
+      <c r="D7" s="7"/>
+      <c r="I7" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="J7" s="7"/>
+      <c r="K7" s="7"/>
+      <c r="Q7" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="R7" s="7"/>
+      <c r="S7" s="7"/>
+    </row>
+    <row r="8" spans="2:19">
+      <c r="B8" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C8" s="7"/>
+      <c r="D8" s="7"/>
+      <c r="Q8" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="R8" s="7"/>
+      <c r="S8" s="7"/>
+    </row>
+    <row r="9" spans="2:19">
+      <c r="I9" s="3"/>
+      <c r="Q9" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="R9" s="7"/>
+      <c r="S9" s="7"/>
+    </row>
+    <row r="10" spans="2:19">
+      <c r="B10" s="2"/>
+      <c r="I10" s="3"/>
+    </row>
+    <row r="11" spans="2:19">
+      <c r="B11" s="2"/>
+      <c r="I11" s="3"/>
+    </row>
+    <row r="12" spans="2:19">
+      <c r="B12" s="3"/>
+      <c r="I12" s="3"/>
+    </row>
+    <row r="13" spans="2:19">
+      <c r="B13" s="3"/>
+      <c r="I13" s="3"/>
+    </row>
+    <row r="14" spans="2:19">
+      <c r="B14" s="3"/>
+      <c r="I14" s="2"/>
+    </row>
+    <row r="15" spans="2:19">
+      <c r="B15" s="2"/>
+      <c r="I15" s="3"/>
+    </row>
+    <row r="16" spans="2:19">
+      <c r="B16" s="3"/>
+      <c r="I16" s="3"/>
+    </row>
+    <row r="17" spans="2:9">
+      <c r="B17" s="2"/>
+      <c r="I17" s="3"/>
+    </row>
+    <row r="18" spans="2:9">
+      <c r="B18" s="2"/>
+      <c r="I18" s="3"/>
+    </row>
+    <row r="19" spans="2:9">
+      <c r="I19" s="2"/>
+    </row>
+    <row r="20" spans="2:9">
+      <c r="I20" s="3"/>
+    </row>
+    <row r="21" spans="2:9">
+      <c r="I21" s="3"/>
+    </row>
+    <row r="22" spans="2:9">
+      <c r="I22" s="2"/>
+    </row>
+    <row r="23" spans="2:9">
+      <c r="I23" s="3"/>
+    </row>
+    <row r="24" spans="2:9">
+      <c r="I24" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
[Comp-751] CEB summary report tweaks
</commit_message>
<xml_diff>
--- a/compliance-api/src/compliance_api/services/report/ceb_template.xlsx
+++ b/compliance-api/src/compliance_api/services/report/ceb_template.xlsx
@@ -1,31 +1,31 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30023"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30110"/>
   <workbookPr hidePivotFieldList="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tayalee/Desktop/Excel pivot tables_forfeedback/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{006F340F-4539-428D-9C2A-553C09694AAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E2829F5B-EA5D-4A74-82D1-896F1117A789}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="35080" yWindow="1540" windowWidth="34560" windowHeight="20260" firstSheet="3" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="35080" yWindow="1540" windowWidth="34560" windowHeight="20260" firstSheet="3" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Inspections" sheetId="13" r:id="rId1"/>
     <sheet name="Requirements" sheetId="11" r:id="rId2"/>
     <sheet name="Enforcement" sheetId="12" r:id="rId3"/>
-    <sheet name="InsightsInsights" sheetId="3" r:id="rId4"/>
+    <sheet name="InspectionInsights" sheetId="3" r:id="rId4"/>
     <sheet name="Complaints" sheetId="14" r:id="rId5"/>
     <sheet name="ComplaintsInsights" sheetId="15" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191028"/>
   <pivotCaches>
-    <pivotCache cacheId="501" r:id="rId7"/>
-    <pivotCache cacheId="509" r:id="rId8"/>
-    <pivotCache cacheId="515" r:id="rId9"/>
-    <pivotCache cacheId="525" r:id="rId10"/>
+    <pivotCache cacheId="1364" r:id="rId7"/>
+    <pivotCache cacheId="1370" r:id="rId8"/>
+    <pivotCache cacheId="1378" r:id="rId9"/>
+    <pivotCache cacheId="1382" r:id="rId10"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -281,7 +281,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -298,24 +298,16 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="25">
+  <dxfs count="23">
     <dxf>
       <fill>
         <patternFill patternType="none">
           <fgColor indexed="64"/>
           <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="3"/>
         </patternFill>
       </fill>
     </dxf>
@@ -335,20 +327,17 @@
     </dxf>
     <dxf>
       <fill>
-        <patternFill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
           <bgColor theme="4" tint="0.39997558519241921"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
-        <patternFill patternType="none"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
         <patternFill patternType="solid">
-          <bgColor theme="3"/>
+          <fgColor indexed="64"/>
+          <bgColor theme="4" tint="0.39997558519241921"/>
         </patternFill>
       </fill>
     </dxf>
@@ -368,52 +357,8 @@
     </dxf>
     <dxf>
       <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
         <patternFill patternType="solid">
-          <bgColor theme="3"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="3"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.39997558519241921"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
           <bgColor theme="4" tint="0.39997558519241921"/>
         </patternFill>
       </fill>
@@ -421,6 +366,7 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
+          <fgColor indexed="64"/>
           <bgColor theme="4" tint="0.39997558519241921"/>
         </patternFill>
       </fill>
@@ -428,6 +374,23 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="4" tint="0.39997558519241921"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="4" tint="0.39997558519241921"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
           <bgColor theme="4" tint="0.39997558519241921"/>
         </patternFill>
       </fill>
@@ -474,6 +437,43 @@
         </patternFill>
       </fill>
     </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.39997558519241921"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.39997558519241921"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor theme="4" tint="0.39997558519241921"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="4" tint="0.39997558519241921"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="4" tint="0.39997558519241921"/>
+        </patternFill>
+      </fill>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -488,184 +488,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshOnLoad="1" refreshedBy="Excel Services" refreshedDate="46148.598844328706" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="1" xr:uid="{9A655F1F-804E-4F57-A400-987732F35DAD}">
-  <cacheSource type="worksheet">
-    <worksheetSource name="Inspections"/>
-  </cacheSource>
-  <cacheFields count="8">
-    <cacheField name="IR Number" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
-    </cacheField>
-    <cacheField name="IR Progress" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1" count="1">
-        <m/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="Project Name" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
-    </cacheField>
-    <cacheField name="Project Type" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
-    </cacheField>
-    <cacheField name="IR Issuance Date" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
-    </cacheField>
-    <cacheField name="Primary Officer" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
-    </cacheField>
-    <cacheField name="Inspection Status" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
-    </cacheField>
-    <cacheField name="Case File Number" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
-    </cacheField>
-  </cacheFields>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
-      <x14:pivotCacheDefinition/>
-    </ext>
-  </extLst>
-</pivotCacheDefinition>
-</file>
-
-<file path=xl/pivotCache/pivotCacheDefinition2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshOnLoad="1" refreshedBy="Excel Services" refreshedDate="46148.598844328706" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="1" xr:uid="{3DC42666-42A1-448D-A623-A82BC44CBAFC}">
-  <cacheSource type="worksheet">
-    <worksheetSource name="Enforcement"/>
-  </cacheSource>
-  <cacheFields count="14">
-    <cacheField name="IR Number" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
-    </cacheField>
-    <cacheField name="IR Progress" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
-    </cacheField>
-    <cacheField name="Project Name" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1" count="1">
-        <m/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="Project Type" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
-    </cacheField>
-    <cacheField name="Compliance Finding" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1" count="1">
-        <m/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="Enforcement Action" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1" count="1">
-        <m/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="Enforcement Status" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1" count="1">
-        <m/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="Enforcement Document Number" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1" count="1">
-        <m/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="IR Issuance Date" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
-    </cacheField>
-    <cacheField name="Primary Officer" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
-    </cacheField>
-    <cacheField name="Inspection Status" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
-    </cacheField>
-    <cacheField name="Case File Number" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
-    </cacheField>
-    <cacheField name="Index" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
-    </cacheField>
-    <cacheField name="Unique Key" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
-    </cacheField>
-  </cacheFields>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
-      <x14:pivotCacheDefinition/>
-    </ext>
-  </extLst>
-</pivotCacheDefinition>
-</file>
-
-<file path=xl/pivotCache/pivotCacheDefinition3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshOnLoad="1" refreshedBy="Excel Services" refreshedDate="46148.598844328706" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="1" xr:uid="{E508D2FB-1B6C-4B04-92EF-07C92A3B7FD7}">
-  <cacheSource type="worksheet">
-    <worksheetSource name="Requirements"/>
-  </cacheSource>
-  <cacheFields count="16">
-    <cacheField name="IR Number" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
-    </cacheField>
-    <cacheField name="Topic" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
-    </cacheField>
-    <cacheField name="Summary" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
-    </cacheField>
-    <cacheField name="IR Progress" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
-    </cacheField>
-    <cacheField name="Project Name" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1" count="1">
-        <m/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="Project Type" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1" count="1">
-        <m/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="Compliance Finding" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1" count="1">
-        <m/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="Enforcement Action" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
-    </cacheField>
-    <cacheField name="Enforcement Status" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
-    </cacheField>
-    <cacheField name="Enforcement Document Number" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
-    </cacheField>
-    <cacheField name="Condition Number" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
-    </cacheField>
-    <cacheField name="Requirement Source" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
-    </cacheField>
-    <cacheField name="IR Issuance Date" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
-    </cacheField>
-    <cacheField name="Primary Officer" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
-    </cacheField>
-    <cacheField name="Inspection Status" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
-    </cacheField>
-    <cacheField name="Case File Number" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
-    </cacheField>
-  </cacheFields>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
-      <x14:pivotCacheDefinition/>
-    </ext>
-  </extLst>
-</pivotCacheDefinition>
-</file>
-
-<file path=xl/pivotCache/pivotCacheDefinition4.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshOnLoad="1" refreshedBy="Excel Services" refreshedDate="46148.598844328706" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="1" xr:uid="{489B308B-C5F1-4496-9EA3-999C745CB76D}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshOnLoad="1" refreshedBy="Excel Services" refreshedDate="46154.646372337964" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="1" xr:uid="{489B308B-C5F1-4496-9EA3-999C745CB76D}">
   <cacheSource type="worksheet">
     <worksheetSource name="Complaints"/>
   </cacheSource>
@@ -726,35 +549,194 @@
 </pivotCacheDefinition>
 </file>
 
+<file path=xl/pivotCache/pivotCacheDefinition2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshOnLoad="1" refreshedBy="Excel Services" refreshedDate="46154.646372337964" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="1" xr:uid="{E508D2FB-1B6C-4B04-92EF-07C92A3B7FD7}">
+  <cacheSource type="worksheet">
+    <worksheetSource name="Requirements"/>
+  </cacheSource>
+  <cacheFields count="16">
+    <cacheField name="IR Number" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="Topic" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="Summary" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="IR Progress" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="Project Name" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1" count="1">
+        <m/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Project Type" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1" count="1">
+        <m/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Compliance Finding" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1" count="1">
+        <m/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Enforcement Action" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="Enforcement Status" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="Enforcement Document Number" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="Condition Number" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="Requirement Source" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="IR Issuance Date" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="Primary Officer" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="Inspection Status" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="Case File Number" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+  </cacheFields>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
+      <x14:pivotCacheDefinition/>
+    </ext>
+  </extLst>
+</pivotCacheDefinition>
+</file>
+
+<file path=xl/pivotCache/pivotCacheDefinition3.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshOnLoad="1" refreshedBy="Excel Services" refreshedDate="46154.646372569441" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="1" xr:uid="{3DC42666-42A1-448D-A623-A82BC44CBAFC}">
+  <cacheSource type="worksheet">
+    <worksheetSource name="Enforcement"/>
+  </cacheSource>
+  <cacheFields count="14">
+    <cacheField name="IR Number" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="IR Progress" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="Project Name" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1" count="1">
+        <m/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Project Type" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="Compliance Finding" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1" count="1">
+        <m/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Enforcement Action" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1" count="1">
+        <m/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Enforcement Status" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1" count="1">
+        <m/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Enforcement Document Number" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1" count="1">
+        <m/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="IR Issuance Date" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="Primary Officer" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="Inspection Status" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="Case File Number" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="Index" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="Unique Key" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+  </cacheFields>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
+      <x14:pivotCacheDefinition/>
+    </ext>
+  </extLst>
+</pivotCacheDefinition>
+</file>
+
+<file path=xl/pivotCache/pivotCacheDefinition4.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshOnLoad="1" refreshedBy="Excel Services" refreshedDate="46154.646372569441" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="1" xr:uid="{9A655F1F-804E-4F57-A400-987732F35DAD}">
+  <cacheSource type="worksheet">
+    <worksheetSource name="Inspections"/>
+  </cacheSource>
+  <cacheFields count="8">
+    <cacheField name="IR Number" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="IR Progress" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1" count="1">
+        <m/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Project Name" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="Project Type" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="IR Issuance Date" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="Primary Officer" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="Inspection Status" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="Case File Number" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+  </cacheFields>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
+      <x14:pivotCacheDefinition/>
+    </ext>
+  </extLst>
+</pivotCacheDefinition>
+</file>
+
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{3A2CB471-5EA6-4127-A467-E8F5D9596452}" name="PivotTable23" cacheId="515" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="E4:G7" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
-  <pivotFields count="16">
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{DE23F307-6508-443D-9D35-8D0EAB9E4958}" name="PivotTable22" cacheId="1382" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="B4:C6" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="8">
     <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
     <pivotField axis="axisRow" showAll="0">
       <items count="2">
         <item x="0"/>
         <item t="default"/>
       </items>
     </pivotField>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="2">
-        <item sd="0" x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField axis="axisCol" showAll="0">
-      <items count="2">
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
@@ -762,9 +744,8 @@
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
   </pivotFields>
-  <rowFields count="2">
-    <field x="5"/>
-    <field x="4"/>
+  <rowFields count="1">
+    <field x="1"/>
   </rowFields>
   <rowItems count="2">
     <i>
@@ -774,38 +755,18 @@
       <x/>
     </i>
   </rowItems>
-  <colFields count="1">
-    <field x="6"/>
-  </colFields>
-  <colItems count="2">
-    <i>
-      <x/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
+  <colItems count="1">
+    <i/>
   </colItems>
   <dataFields count="1">
-    <dataField name="Count of Summary" fld="2" subtotal="count" baseField="0" baseItem="0"/>
+    <dataField name="Count of IR Number" fld="0" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
-  <formats count="6">
-    <format dxfId="19">
-      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="20">
-      <pivotArea field="6" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
-    </format>
+  <formats count="2">
     <format dxfId="21">
-      <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
     <format dxfId="22">
-      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="23">
-      <pivotArea field="6" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
-    </format>
-    <format dxfId="24">
-      <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+      <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
   </formats>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
@@ -821,54 +782,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{DE23F307-6508-443D-9D35-8D0EAB9E4958}" name="PivotTable22" cacheId="501" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="B4:C6" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="8">
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="2">
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="1"/>
-  </rowFields>
-  <rowItems count="2">
-    <i>
-      <x/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Count of IR Number" fld="0" subtotal="count" baseField="0" baseItem="0"/>
-  </dataFields>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{F3646FCF-C206-4361-8690-240132D1671E}" name="PivotTable24" cacheId="509" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{F3646FCF-C206-4361-8690-240132D1671E}" name="PivotTable24" cacheId="1378" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="K6:M11" firstHeaderRow="1" firstDataRow="2" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="14">
     <pivotField showAll="0"/>
@@ -948,13 +862,13 @@
     <dataField name="Count of Enforcement Action" fld="5" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="3">
-    <format dxfId="16">
+    <format dxfId="18">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="17">
+    <format dxfId="19">
       <pivotArea field="6" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="18">
+    <format dxfId="20">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -970,8 +884,102 @@
 </pivotTableDefinition>
 </file>
 
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{3A2CB471-5EA6-4127-A467-E8F5D9596452}" name="PivotTable23" cacheId="1370" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="E4:G7" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="16">
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="2">
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="2">
+        <item sd="0" x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisCol" showAll="0">
+      <items count="2">
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="2">
+    <field x="5"/>
+    <field x="4"/>
+  </rowFields>
+  <rowItems count="2">
+    <i>
+      <x/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="6"/>
+  </colFields>
+  <colItems count="2">
+    <i>
+      <x/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Count of Summary" fld="2" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <formats count="6">
+    <format dxfId="12">
+      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="13">
+      <pivotArea field="6" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
+    </format>
+    <format dxfId="14">
+      <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="15">
+      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="16">
+      <pivotArea field="6" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
+    </format>
+    <format dxfId="17">
+      <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+    </format>
+  </formats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
 <file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{49EF033C-CFA8-44B9-BC70-D0C253FFC2B0}" name="Project Complaints by Topic and Resolution" cacheId="525" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{49EF033C-CFA8-44B9-BC70-D0C253FFC2B0}" name="Project Complaints by Topic and Resolution" cacheId="1364" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="Q4:S9" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="11">
     <pivotField axis="axisRow" showAll="0">
@@ -1039,20 +1047,14 @@
   <dataFields count="1">
     <dataField name="Count of Complaint Resolution" fld="9" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
-  <formats count="5">
-    <format dxfId="11">
+  <formats count="3">
+    <format dxfId="9">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="12">
-      <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+    <format dxfId="10">
+      <pivotArea field="9" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
-    <format dxfId="13">
-      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="14">
-      <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="15">
+    <format dxfId="11">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -1069,7 +1071,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{4DC00558-9D6A-4D8C-A8BC-4CABB5BCD879}" name="Complaint Sources by Project" cacheId="525" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{4DC00558-9D6A-4D8C-A8BC-4CABB5BCD879}" name="Complaint Sources by Project" cacheId="1364" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="I4:K7" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="11">
     <pivotField showAll="0"/>
@@ -1125,20 +1127,17 @@
   <dataFields count="1">
     <dataField name="Count of Complaint Source" fld="5" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
-  <formats count="5">
+  <formats count="4">
+    <format dxfId="5">
+      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+    </format>
     <format dxfId="6">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
     <format dxfId="7">
-      <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+      <pivotArea field="5" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
     <format dxfId="8">
-      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="9">
-      <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="10">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -1155,7 +1154,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{A78A3DE9-337B-4375-ABAF-39D54018E350}" name="Complaint Source and Resolution Summary" cacheId="525" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{A78A3DE9-337B-4375-ABAF-39D54018E350}" name="Complaint Source and Resolution Summary" cacheId="1364" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="B4:D8" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="11">
     <pivotField dataField="1" showAll="0"/>
@@ -1214,20 +1213,17 @@
   <dataFields count="1">
     <dataField name="Count of Complaint Number" fld="0" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
-  <formats count="5">
+  <formats count="4">
     <format dxfId="1">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
     <format dxfId="2">
-      <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
     <format dxfId="3">
-      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+      <pivotArea field="9" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
     <format dxfId="4">
-      <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="5">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -1911,10 +1907,10 @@
       </c>
     </row>
     <row r="4" spans="2:13">
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="4" t="s">
         <v>22</v>
       </c>
       <c r="E4" s="4" t="s">
@@ -2106,24 +2102,24 @@
       <c r="B4" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="D4" s="8"/>
+      <c r="D4" s="4"/>
       <c r="I4" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="J4" s="1" t="s">
+      <c r="J4" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="K4" s="8"/>
+      <c r="K4" s="4"/>
       <c r="Q4" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="R4" s="1" t="s">
+      <c r="R4" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="S4" s="8"/>
+      <c r="S4" s="4"/>
     </row>
     <row r="5" spans="2:19">
       <c r="B5" s="1" t="s">

</xml_diff>